<commit_message>
Expand hardware database with Ampere CPUs, used servers, and SSDs
</commit_message>
<xml_diff>
--- a/hardware_database.xlsx
+++ b/hardware_database.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc179c94a123f4525"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="2" r:id="Re33dba4cdc034438"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="3" r:id="R6178804635494d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile SoC" sheetId="4" r:id="R01b1bbb29a134584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoM" sheetId="5" r:id="R6f5514a19c4648b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accelerator" sheetId="6" r:id="Rc247c8b114c64536"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform" sheetId="7" r:id="Rfea4bf48c7d742a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0ac5f4880bd94723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="2" r:id="Ra5fcb9dac2184af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="3" r:id="R19728180de0f4bdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile SoC" sheetId="4" r:id="R2378b094c2a44659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoM" sheetId="5" r:id="Rc83407632c574e22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accelerator" sheetId="6" r:id="Re05c6a58b5f44467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform" sheetId="7" r:id="R13bf758629fa4f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="8" r:id="Ra4dc11171ccb445e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,13 +20,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="10">
     <x:numFmt numFmtId="200" formatCode="&quot;$&quot;#,##0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
     <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="204" formatCode="$#,##0"/>
+    <x:numFmt numFmtId="205" formatCode="$#,##0.00"/>
+    <x:numFmt numFmtId="206" formatCode="0"/>
+    <x:numFmt numFmtId="207" formatCode="0.000"/>
+    <x:numFmt numFmtId="208" formatCode="0.0"/>
+    <x:numFmt numFmtId="209" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -76,8 +83,41 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF263445"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF19395C"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF19395C"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF5A6472"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF0563C1"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF5A6472"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -99,8 +139,63 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19395C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19395C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border>
       <x:left/>
       <x:right/>
@@ -157,11 +252,20 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="medium">
+        <x:color rgb="FF19395C"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="52">
+  <x:cellXfs count="206">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -280,6 +384,436 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -288,9 +822,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CPUTable" displayName="CPUTable" ref="A6:R14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:R14"/>
-  <x:tableColumns count="18">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="CPUTable" displayName="CPUTable" ref="A6:Y17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:Y17"/>
+  <x:tableColumns count="25">
     <x:tableColumn id="1" name="Vendor"/>
     <x:tableColumn id="2" name="Model"/>
     <x:tableColumn id="3" name="Architecture"/>
@@ -309,6 +843,13 @@
     <x:tableColumn id="16" name="Price date"/>
     <x:tableColumn id="17" name="Source"/>
     <x:tableColumn id="18" name="Notes"/>
+    <x:tableColumn id="19" name="NVMe lanes max at CPU gen (1P)"/>
+    <x:tableColumn id="20" name="x4 SSDs (lane-budget max)"/>
+    <x:tableColumn id="21" name="PCIe per lane (GB/s; one way)"/>
+    <x:tableColumn id="22" name="RAID0 PCIe ceiling (GB/s)"/>
+    <x:tableColumn id="23" name="RAID0 PCIe/RAM ceiling (GB/s)"/>
+    <x:tableColumn id="24" name="NVMe lane / RAID0 constraints"/>
+    <x:tableColumn id="25" name="NVMe lane sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -423,8 +964,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PlatformTable" displayName="PlatformTable" ref="A6:R13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:R13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PlatformTable" displayName="PlatformTable" ref="A6:R16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:R16"/>
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="Vendor"/>
     <x:tableColumn id="2" name="System"/>
@@ -444,6 +985,34 @@
     <x:tableColumn id="16" name="1 TiB system cost (USD)"/>
     <x:tableColumn id="17" name="Source"/>
     <x:tableColumn id="18" name="Notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="SSDTable" displayName="SSDTable" ref="A6:T12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="20">
+    <x:tableColumn id="1" name="Vendor"/>
+    <x:tableColumn id="2" name="Model / part number"/>
+    <x:tableColumn id="3" name="Condition"/>
+    <x:tableColumn id="4" name="Capacity (TB; decimal)"/>
+    <x:tableColumn id="5" name="Form factor"/>
+    <x:tableColumn id="6" name="PCIe generation"/>
+    <x:tableColumn id="7" name="PCIe lanes"/>
+    <x:tableColumn id="8" name="Seq. read up to (MB/s)"/>
+    <x:tableColumn id="9" name="Seq. write up to (MB/s)"/>
+    <x:tableColumn id="10" name="Rated endurance (TBW)"/>
+    <x:tableColumn id="11" name="Power-loss protection"/>
+    <x:tableColumn id="12" name="Price (USD)"/>
+    <x:tableColumn id="13" name="Price basis / seller"/>
+    <x:tableColumn id="14" name="Availability"/>
+    <x:tableColumn id="15" name="Price date"/>
+    <x:tableColumn id="16" name="Price / TB (USD)"/>
+    <x:tableColumn id="17" name="4x RAID0 read (GB/s; ideal)"/>
+    <x:tableColumn id="18" name="4x RAID0 write (GB/s; ideal)"/>
+    <x:tableColumn id="19" name="Sources"/>
+    <x:tableColumn id="20" name="Notes"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -692,7 +1261,7 @@
       </x:c>
       <x:c r="B7" s="47" t="n">
         <x:f>COUNTA('CPU'!A7:A1000)</x:f>
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="47" t="str">
         <x:v>Server, workstation and HBM CPU parts</x:v>
@@ -752,10 +1321,22 @@
       </x:c>
       <x:c r="B12" s="46" t="n">
         <x:f>COUNTA('Platform'!A7:A1000)</x:f>
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C12" s="46" t="str">
         <x:v>Complete systems and server platforms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>SSD</x:v>
+      </x:c>
+      <x:c r="B13" s="47" t="n">
+        <x:f>COUNTA('SSD'!B7:B1000)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>New and used NVMe SSDs, endurance and RAID0 estimates</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -880,6 +1461,13 @@
     <x:col min="16" max="16" width="7.559999942779541" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="52" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="23" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="21" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="23" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="25" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="25" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="64" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="85" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -929,7 +1517,7 @@
       <x:c r="Q4" s="24"/>
       <x:c r="R4" s="24"/>
     </x:row>
-    <x:row r="6" ht="32" hidden="0" customHeight="1">
+    <x:row r="6" ht="48" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
         <x:v>Vendor</x:v>
       </x:c>
@@ -984,8 +1572,29 @@
       <x:c r="R6" s="18" t="str">
         <x:v>Notes</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="S6" s="140" t="str">
+        <x:v>NVMe lanes max at CPU gen (1P)</x:v>
+      </x:c>
+      <x:c r="T6" s="140" t="str">
+        <x:v>x4 SSDs (lane-budget max)</x:v>
+      </x:c>
+      <x:c r="U6" s="140" t="str">
+        <x:v>PCIe per lane (GB/s; one way)</x:v>
+      </x:c>
+      <x:c r="V6" s="140" t="str">
+        <x:v>RAID0 PCIe ceiling (GB/s)</x:v>
+      </x:c>
+      <x:c r="W6" s="140" t="str">
+        <x:v>RAID0 PCIe/RAM ceiling (GB/s)</x:v>
+      </x:c>
+      <x:c r="X6" s="140" t="str">
+        <x:v>NVMe lane / RAID0 constraints</x:v>
+      </x:c>
+      <x:c r="Y6" s="140" t="str">
+        <x:v>NVMe lane sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="60" hidden="0" customHeight="1">
       <x:c r="A7" s="22" t="str">
         <x:v>AMD</x:v>
       </x:c>
@@ -1040,8 +1649,34 @@
       <x:c r="R7" s="22" t="str">
         <x:v>Bandwidth is theoretical at MRDIMM-12800. Max memory is a platform estimate pending a detailed public SKU datasheet.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="S7" s="148" t="n">
+        <x:f>J7</x:f>
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="T7" s="148" t="n">
+        <x:f>INT(S7/4)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="U7" s="149" t="n">
+        <x:f>IF(I7="PCIe 6.0",64/8*236/256,IF(I7="PCIe 5.0",32/8*128/130,IF(I7="PCIe 4.0",16/8*128/130,IF(I7="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>7.375</x:v>
+      </x:c>
+      <x:c r="V7" s="150" t="n">
+        <x:f>T7*4*U7</x:f>
+        <x:v>708</x:v>
+      </x:c>
+      <x:c r="W7" s="150" t="n">
+        <x:f>MIN(V7,H7)</x:f>
+        <x:v>708</x:v>
+      </x:c>
+      <x:c r="X7" s="144" t="str">
+        <x:v>96 Gen6 lanes: conditional CPU budget; board/root-port fan-out unverified. Requires Gen6 SSDs for this ceiling; Gen5 SSDs cap these lanes at 378.1 GB/s.</x:v>
+      </x:c>
+      <x:c r="Y7" s="144" t="str">
+        <x:v>https://www.amd.com/en/products/processors/server/epyc/9006-series/amd-epyc-9996.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="60" hidden="0" customHeight="1">
       <x:c r="A8" s="21" t="str">
         <x:v>AMD</x:v>
       </x:c>
@@ -1096,8 +1731,34 @@
       <x:c r="R8" s="21" t="str">
         <x:v>Six TB DDR5 per socket. AMD also documents up to 2 TB of CXL memory beyond DDR capacity.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="S8" s="158" t="n">
+        <x:f>J8</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="T8" s="158" t="n">
+        <x:f>INT(S8/4)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="U8" s="159" t="n">
+        <x:f>IF(I8="PCIe 6.0",64/8*236/256,IF(I8="PCIe 5.0",32/8*128/130,IF(I8="PCIe 4.0",16/8*128/130,IF(I8="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V8" s="160" t="n">
+        <x:f>T8*4*U8</x:f>
+        <x:v>504.12307692307695</x:v>
+      </x:c>
+      <x:c r="W8" s="160" t="n">
+        <x:f>MIN(V8,H8)</x:f>
+        <x:v>504.12307692307695</x:v>
+      </x:c>
+      <x:c r="X8" s="154" t="str">
+        <x:v>128 Gen5 lanes in 1P, assuming all routed to NVMe. SATA, CXL and other devices share platform resources; 2P routing differs.</x:v>
+      </x:c>
+      <x:c r="Y8" s="154" t="str">
+        <x:v>https://www.amd.com/en/products/processors/server/epyc/9005-series/amd-epyc-9965.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="60" hidden="0" customHeight="1">
       <x:c r="A9" s="23" t="str">
         <x:v>Intel</x:v>
       </x:c>
@@ -1152,8 +1813,34 @@
       <x:c r="R9" s="23" t="str">
         <x:v>844.8 GB/s assumes 12 channels at MRDIMM-8800. DDR5-6400 yields 614.4 GB/s.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="S9" s="148" t="n">
+        <x:f>J9</x:f>
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="T9" s="148" t="n">
+        <x:f>INT(S9/4)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="U9" s="149" t="n">
+        <x:f>IF(I9="PCIe 6.0",64/8*236/256,IF(I9="PCIe 5.0",32/8*128/130,IF(I9="PCIe 4.0",16/8*128/130,IF(I9="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V9" s="150" t="n">
+        <x:f>T9*4*U9</x:f>
+        <x:v>378.0923076923077</x:v>
+      </x:c>
+      <x:c r="W9" s="150" t="n">
+        <x:f>MIN(V9,H9)</x:f>
+        <x:v>378.0923076923077</x:v>
+      </x:c>
+      <x:c r="X9" s="144" t="str">
+        <x:v>96 Gen5 lanes per CPU. Drive count is a lane-budget equivalent; suitable root ports, bifurcation or switches and board wiring required.</x:v>
+      </x:c>
+      <x:c r="Y9" s="144" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/240777/intel-xeon-6980p-processor-504m-cache-2-00-ghz/specifications.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="60" hidden="0" customHeight="1">
       <x:c r="A10" s="21" t="str">
         <x:v>AMD</x:v>
       </x:c>
@@ -1208,8 +1895,34 @@
       <x:c r="R10" s="21" t="str">
         <x:v>CPU price excludes motherboard and twelve or twenty-four DIMMs.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="S10" s="158" t="n">
+        <x:f>J10</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="T10" s="158" t="n">
+        <x:f>INT(S10/4)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="U10" s="159" t="n">
+        <x:f>IF(I10="PCIe 6.0",64/8*236/256,IF(I10="PCIe 5.0",32/8*128/130,IF(I10="PCIe 4.0",16/8*128/130,IF(I10="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V10" s="160" t="n">
+        <x:f>T10*4*U10</x:f>
+        <x:v>504.12307692307695</x:v>
+      </x:c>
+      <x:c r="W10" s="160" t="n">
+        <x:f>MIN(V10,H10)</x:f>
+        <x:v>460.8</x:v>
+      </x:c>
+      <x:c r="X10" s="154" t="str">
+        <x:v>128 Gen5 lanes in 1P, assuming all routed to NVMe. Platform SATA/other I/O reduces available lanes; 2P routing differs.</x:v>
+      </x:c>
+      <x:c r="Y10" s="154" t="str">
+        <x:v>https://www.amd.com/en/products/processors/server/epyc/4th-generation-9004-and-8004-series/amd-epyc-9654.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="60" hidden="0" customHeight="1">
       <x:c r="A11" s="23" t="str">
         <x:v>AMD</x:v>
       </x:c>
@@ -1264,8 +1977,35 @@
       <x:c r="R11" s="23" t="str">
         <x:v>Workstation platform. Maximum capacity depends on the WRX90 motherboard and supported RDIMMs.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="S11" s="148" t="n">
+        <x:f>J11</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="T11" s="148" t="n">
+        <x:f>INT(S11/4)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="U11" s="149" t="n">
+        <x:f>IF(I11="PCIe 6.0",64/8*236/256,IF(I11="PCIe 5.0",32/8*128/130,IF(I11="PCIe 4.0",16/8*128/130,IF(I11="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V11" s="150" t="n">
+        <x:f>T11*4*U11</x:f>
+        <x:v>504.12307692307695</x:v>
+      </x:c>
+      <x:c r="W11" s="150" t="n">
+        <x:f>MIN(V11,H11)</x:f>
+        <x:v>409.6</x:v>
+      </x:c>
+      <x:c r="X11" s="144" t="str">
+        <x:v>128 Gen5 lanes only, on WRX90; excludes slower chipset lanes sharing their uplink. TRX50 exposes fewer lanes; subtract board NIC/GPU allocations.</x:v>
+      </x:c>
+      <x:c r="Y11" s="144" t="str">
+        <x:v>https://www.amd.com/en/products/processors/workstations/ryzen-threadripper/9000-wx-series/amd-ryzen-threadripper-pro-9995wx.html
+https://www.asus.com/motherboards-components/motherboards/workstation/pro-ws-wrx90e-sage-se/techspec/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="60" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
         <x:v>Intel</x:v>
       </x:c>
@@ -1320,8 +2060,34 @@
       <x:c r="R12" s="21" t="str">
         <x:v>Vendor RCP was much higher. Recheck current distributor stock before purchase.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="S12" s="158" t="n">
+        <x:f>J12</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="T12" s="158" t="n">
+        <x:f>INT(S12/4)</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="U12" s="159" t="n">
+        <x:f>IF(I12="PCIe 6.0",64/8*236/256,IF(I12="PCIe 5.0",32/8*128/130,IF(I12="PCIe 4.0",16/8*128/130,IF(I12="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V12" s="160" t="n">
+        <x:f>T12*4*U12</x:f>
+        <x:v>315.0769230769231</x:v>
+      </x:c>
+      <x:c r="W12" s="160" t="n">
+        <x:f>MIN(V12,H12)</x:f>
+        <x:v>315.0769230769231</x:v>
+      </x:c>
+      <x:c r="X12" s="154" t="str">
+        <x:v>80 Gen5 lanes per CPU; all-NVMe CPU budget, subject to board/root-port topology. Software RAID0 can span controllers; firmware RAID limits vary.</x:v>
+      </x:c>
+      <x:c r="Y12" s="154" t="str">
+        <x:v>https://www.intel.com/content/www/us/en/products/sku/237261/intel-xeon-platinum-8592-processor-320m-cache-1-90-ghz/specifications.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="60" hidden="0" customHeight="1">
       <x:c r="A13" s="23" t="str">
         <x:v>AMD</x:v>
       </x:c>
@@ -1376,8 +2142,34 @@
       <x:c r="R13" s="23" t="str">
         <x:v>Used price varies strongly with locking status and seller testing.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="S13" s="148" t="n">
+        <x:f>J13</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="T13" s="148" t="n">
+        <x:f>INT(S13/4)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="U13" s="149" t="n">
+        <x:f>IF(I13="PCIe 6.0",64/8*236/256,IF(I13="PCIe 5.0",32/8*128/130,IF(I13="PCIe 4.0",16/8*128/130,IF(I13="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>1.9692307692307693</x:v>
+      </x:c>
+      <x:c r="V13" s="150" t="n">
+        <x:f>T13*4*U13</x:f>
+        <x:v>252.06153846153848</x:v>
+      </x:c>
+      <x:c r="W13" s="150" t="n">
+        <x:f>MIN(V13,H13)</x:f>
+        <x:v>204.8</x:v>
+      </x:c>
+      <x:c r="X13" s="144" t="str">
+        <x:v>128 Gen4 lanes in 1P; shared platform I/O reduces storage lanes. 2P uses I/O resources for inter-socket links. RAM ceiling below PCIe ceiling.</x:v>
+      </x:c>
+      <x:c r="Y13" s="144" t="str">
+        <x:v>https://www.amd.com/ja/support/downloads/drivers.html/processors/epyc/epyc-7002-series/amd-epyc-7742.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="60" hidden="0" customHeight="1">
       <x:c r="A14" s="21" t="str">
         <x:v>Fujitsu</x:v>
       </x:c>
@@ -1428,11 +2220,382 @@
       <x:c r="R14" s="21" t="str">
         <x:v>HBM capacity is fixed. PCIe is primarily for I/O rather than large accelerator fan-out.</x:v>
       </x:c>
+      <x:c r="S14" s="158" t="n">
+        <x:f>J14</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="T14" s="158" t="n">
+        <x:f>INT(S14/4)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U14" s="159" t="n">
+        <x:f>IF(I14="PCIe 6.0",64/8*236/256,IF(I14="PCIe 5.0",32/8*128/130,IF(I14="PCIe 4.0",16/8*128/130,IF(I14="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>0.9846153846153847</x:v>
+      </x:c>
+      <x:c r="V14" s="160" t="n">
+        <x:f>T14*4*U14</x:f>
+        <x:v>15.753846153846155</x:v>
+      </x:c>
+      <x:c r="W14" s="160" t="n">
+        <x:f>MIN(V14,H14)</x:f>
+        <x:v>15.753846153846155</x:v>
+      </x:c>
+      <x:c r="X14" s="154" t="str">
+        <x:v>16 Gen3 lanes total; 4 x4 SSDs are a switched fan-out equivalent, not verified direct ports. A64FX system may reserve link for fabric/NIC; NVMe availability unverified.</x:v>
+      </x:c>
+      <x:c r="Y14" s="154" t="str">
+        <x:v>https://global.fujitsu/ja-JP/technology/research/fugaku/specifications</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="120" customHeight="1">
+      <x:c r="A15" s="65" t="str">
+        <x:v>Ampere</x:v>
+      </x:c>
+      <x:c r="B15" s="65" t="str">
+        <x:v>AmpereOne M A192-32M</x:v>
+      </x:c>
+      <x:c r="C15" s="65" t="str">
+        <x:v>Armv8.6+; 192 cores at 3.2 GHz</x:v>
+      </x:c>
+      <x:c r="D15" s="65" t="str">
+        <x:v>DDR5 ECC RDIMM</x:v>
+      </x:c>
+      <x:c r="E15" s="66" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F15" s="66" t="n">
+        <x:v>5600</x:v>
+      </x:c>
+      <x:c r="G15" s="66" t="n">
+        <x:v>1536</x:v>
+      </x:c>
+      <x:c r="H15" s="67" t="n">
+        <x:f>E15*F15*8/1000</x:f>
+        <x:v>537.6</x:v>
+      </x:c>
+      <x:c r="I15" s="65" t="str">
+        <x:v>PCIe 5.0</x:v>
+      </x:c>
+      <x:c r="J15" s="66" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="K15" s="65" t="str">
+        <x:v>FCLGA7228</x:v>
+      </x:c>
+      <x:c r="L15" s="66" t="n">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="M15" s="68" t="n">
+        <x:v>5119</x:v>
+      </x:c>
+      <x:c r="N15" s="65" t="str">
+        <x:v>DataBit listed price; out of stock</x:v>
+      </x:c>
+      <x:c r="O15" s="65" t="str">
+        <x:v>Launched; listed seller out of stock</x:v>
+      </x:c>
+      <x:c r="P15" s="77" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q15" s="70" t="str">
+        <x:v>Specs: https://amperecomputing.com/en/briefs/ampereone-m-product-brief
+Price: https://shop.databitinc.com/Products/overview/M026114271
+TDP (CPU QVL): https://www.gigabyte.com/Enterprise/Rack-Server/R2A3-T40-AAV1/Support-QVL</x:v>
+      </x:c>
+      <x:c r="R15" s="65" t="str">
+        <x:v>1 DIMM/channel. Capacity uses 1024 GB/TB. TDP: 425 W, explicitly listed for A192-32M in GIGABYTE R2A3-T40-AAV1 CPU QVL (updated 2026-03-05; checked 2026-10-18). Ampere’s 348 W is benchmark usage power, not TDP. Price is for AC-S40070; excludes RAM and platform.</x:v>
+      </x:c>
+      <x:c r="S15" s="148" t="n">
+        <x:f>J15</x:f>
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="T15" s="148" t="n">
+        <x:f>INT(S15/4)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="U15" s="149" t="n">
+        <x:f>IF(I15="PCIe 6.0",64/8*236/256,IF(I15="PCIe 5.0",32/8*128/130,IF(I15="PCIe 4.0",16/8*128/130,IF(I15="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V15" s="150" t="n">
+        <x:f>T15*4*U15</x:f>
+        <x:v>378.0923076923077</x:v>
+      </x:c>
+      <x:c r="W15" s="150" t="n">
+        <x:f>MIN(V15,H15)</x:f>
+        <x:v>378.0923076923077</x:v>
+      </x:c>
+      <x:c r="X15" s="144" t="str">
+        <x:v>96 Gen5 lanes; 24 controllers, bifurcation down to x4. 24 x4 SSDs require board/backplane exposing every controller; subtract NIC/other I/O.</x:v>
+      </x:c>
+      <x:c r="Y15" s="144" t="str">
+        <x:v>https://amperecomputing.com/en/briefs/ampereone-m-product-brief</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="120" customHeight="1">
+      <x:c r="A16" s="71" t="str">
+        <x:v>Ampere</x:v>
+      </x:c>
+      <x:c r="B16" s="71" t="str">
+        <x:v>AmpereOne A192-32X</x:v>
+      </x:c>
+      <x:c r="C16" s="71" t="str">
+        <x:v>Armv8.6+; 192 cores at 3.2 GHz</x:v>
+      </x:c>
+      <x:c r="D16" s="71" t="str">
+        <x:v>DDR5 ECC RDIMM</x:v>
+      </x:c>
+      <x:c r="E16" s="72" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F16" s="72" t="n">
+        <x:v>5200</x:v>
+      </x:c>
+      <x:c r="G16" s="72" t="n">
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="H16" s="73" t="n">
+        <x:f>E16*F16*8/1000</x:f>
+        <x:v>332.8</x:v>
+      </x:c>
+      <x:c r="I16" s="71" t="str">
+        <x:v>PCIe 5.0</x:v>
+      </x:c>
+      <x:c r="J16" s="72" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="K16" s="71" t="str">
+        <x:v>FCLGA5964</x:v>
+      </x:c>
+      <x:c r="L16" s="72" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="M16" s="74" t="n">
+        <x:v>5770</x:v>
+      </x:c>
+      <x:c r="N16" s="71" t="str">
+        <x:v>NeweggBusiness listed; out of stock</x:v>
+      </x:c>
+      <x:c r="O16" s="71" t="str">
+        <x:v>Launched; listed seller out of stock</x:v>
+      </x:c>
+      <x:c r="P16" s="78" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q16" s="76" t="str">
+        <x:v>Specs: https://amperecomputing.com/en/briefs/ampereone-family-product-brief
+Price: https://www.neweggbusiness.com/ampereone-a192-32x-3-2ghz-192-core-276w-lga-5964/p/9B-19-999-013
+TDP (CPU QVL): https://www.gigabyte.com/ie/Enterprise/Rack-Server/R163-P32-AAH1/Support-QVL</x:v>
+      </x:c>
+      <x:c r="R16" s="71" t="str">
+        <x:v>1 or 2 DIMMs/channel; maximum speed depends on DIMM population. Capacity uses 1024 GB/TB. TDP: 400 W, explicitly listed for A192-32X in GIGABYTE R163-P32-AAH1 CPU QVL (updated 2026-06-28; checked 2026-10-18). Ampere’s 283 W is benchmark usage power, not TDP. Price excludes RAM and platform.</x:v>
+      </x:c>
+      <x:c r="S16" s="158" t="n">
+        <x:f>J16</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="T16" s="158" t="n">
+        <x:f>INT(S16/4)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="U16" s="159" t="n">
+        <x:f>IF(I16="PCIe 6.0",64/8*236/256,IF(I16="PCIe 5.0",32/8*128/130,IF(I16="PCIe 4.0",16/8*128/130,IF(I16="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>3.9384615384615387</x:v>
+      </x:c>
+      <x:c r="V16" s="160" t="n">
+        <x:f>T16*4*U16</x:f>
+        <x:v>504.12307692307695</x:v>
+      </x:c>
+      <x:c r="W16" s="160" t="n">
+        <x:f>MIN(V16,H16)</x:f>
+        <x:v>332.8</x:v>
+      </x:c>
+      <x:c r="X16" s="154" t="str">
+        <x:v>128 Gen5 lanes in 1P; 32 controllers, x4 fan-out. 32 x4 SSDs require full board exposure. Reserve lanes for NICs; multi-socket topology differs.</x:v>
+      </x:c>
+      <x:c r="Y16" s="154" t="str">
+        <x:v>https://amperecomputing.com/en/briefs/ampereone-family-product-brief</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="120" customHeight="1">
+      <x:c r="A17" s="79" t="str">
+        <x:v>Ampere</x:v>
+      </x:c>
+      <x:c r="B17" s="79" t="str">
+        <x:v>Altra Max M128-30</x:v>
+      </x:c>
+      <x:c r="C17" s="79" t="str">
+        <x:v>Armv8.2+; 128 cores at 3.0 GHz</x:v>
+      </x:c>
+      <x:c r="D17" s="79" t="str">
+        <x:v>DDR4 ECC RDIMM / LRDIMM</x:v>
+      </x:c>
+      <x:c r="E17" s="80" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F17" s="80" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="G17" s="80" t="n">
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="H17" s="81" t="n">
+        <x:f>E17*F17*8/1000</x:f>
+        <x:v>204.8</x:v>
+      </x:c>
+      <x:c r="I17" s="79" t="str">
+        <x:v>PCIe 4.0</x:v>
+      </x:c>
+      <x:c r="J17" s="80" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="K17" s="79" t="str">
+        <x:v>FCLGA4926</x:v>
+      </x:c>
+      <x:c r="L17" s="80" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="M17" s="85" t="n">
+        <x:v>2299.99</x:v>
+      </x:c>
+      <x:c r="N17" s="79" t="str">
+        <x:v>Newegg listed price; out of stock</x:v>
+      </x:c>
+      <x:c r="O17" s="79" t="str">
+        <x:v>Launched; listed seller out of stock</x:v>
+      </x:c>
+      <x:c r="P17" s="83" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q17" s="84" t="str">
+        <x:v>Specs / TDP: Ampere datasheet v1.05, pp. 1, 7, 11: https://d1o0i0v5q5lp8h.cloudfront.net/ampere/live/assets/documents/Altra_Max_Rev_A1_DS_v1.05_20220728.pdf
+Price: https://www.newegg.com/ampere-altra-max-lga-4926/p/N82E16819999002</x:v>
+      </x:c>
+      <x:c r="R17" s="79" t="str">
+        <x:v>128 cores / 128 threads; 1 MB L2/core; 16 MB system cache; TSMC 7 nm. Up to 16 DIMMs (2DPC), 4 TB/socket (4096 GB by table convention). Bandwidth counts 64 data bits/channel, excluding ECC. 128 PCIe lanes in 1P; 2P uses lanes for CCIX (192 external lanes/system). 250 W is SKU TDP, distinct from benchmark usage power. Part AC-212825002; price excludes RAM and platform.</x:v>
+      </x:c>
+      <x:c r="S17" s="148" t="n">
+        <x:f>J17</x:f>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="T17" s="148" t="n">
+        <x:f>INT(S17/4)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="U17" s="149" t="n">
+        <x:f>IF(I17="PCIe 6.0",64/8*236/256,IF(I17="PCIe 5.0",32/8*128/130,IF(I17="PCIe 4.0",16/8*128/130,IF(I17="PCIe 3.0",8/8*128/130,""))))</x:f>
+        <x:v>1.9692307692307693</x:v>
+      </x:c>
+      <x:c r="V17" s="150" t="n">
+        <x:f>T17*4*U17</x:f>
+        <x:v>252.06153846153848</x:v>
+      </x:c>
+      <x:c r="W17" s="150" t="n">
+        <x:f>MIN(V17,H17)</x:f>
+        <x:v>204.8</x:v>
+      </x:c>
+      <x:c r="X17" s="144" t="str">
+        <x:v>128 Gen4 lanes / 32 x4 controllers in 1P; 2P provides 192 external lanes total. RAM ceiling below PCIe ceiling; reserve board/NIC lanes.</x:v>
+      </x:c>
+      <x:c r="Y17" s="144" t="str">
+        <x:v>https://d1o0i0v5q5lp8h.cloudfront.net/ampere/live/assets/documents/Altra_Max_Rev_A1_DS_v1.05_20220728.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="S19" s="161" t="str">
+        <x:v>NVMe / RAID0 calculation basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="S20" s="164" t="str">
+        <x:v>Scope: one CPU / single-socket lane budget at the generation in column I. All listed high-speed lanes assigned to NVMe; no GPU/NIC reservation. CPU limits are conditional, not a purchasable board configuration.</x:v>
+      </x:c>
+      <x:c r="T20" s="164"/>
+      <x:c r="U20" s="164"/>
+      <x:c r="V20" s="164"/>
+      <x:c r="W20" s="164"/>
+      <x:c r="X20" s="164"/>
+      <x:c r="Y20" s="164"/>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="S21" s="164" t="str">
+        <x:v>x4 SSD count = floor(lanes / 4), assuming independent full-width links or non-oversubscribed switch fan-out. More drives behind a switch do not raise upstream bandwidth. No specific SSD model is assumed.</x:v>
+      </x:c>
+      <x:c r="T21" s="164"/>
+      <x:c r="U21" s="164"/>
+      <x:c r="V21" s="164"/>
+      <x:c r="W21" s="164"/>
+      <x:c r="X21" s="164"/>
+      <x:c r="Y21" s="164"/>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="S22" s="164" t="str">
+        <x:v>Per-lane rates: Gen3/4/5 = 8/16/32 GT/s × 128/130 ÷ 8. Gen6 = 64 Gb/s ÷ 8 × 236/256 TLP-byte fraction. Decimal GB/s, one direction; additional packet/NVMe overhead is excluded.</x:v>
+      </x:c>
+      <x:c r="T22" s="164"/>
+      <x:c r="U22" s="164"/>
+      <x:c r="V22" s="164"/>
+      <x:c r="W22" s="164"/>
+      <x:c r="X22" s="164"/>
+      <x:c r="Y22" s="164"/>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="S23" s="164" t="str">
+        <x:v>For host-memory transfers: RAID0 PCIe ceiling = x4 drive count × 4 × per-lane rate. PCIe/RAM ceiling = MIN(PCIe ceiling, peak memory bandwidth in H). Both are theoretical upper bounds; actual read/write speeds depend on SSDs, memory traffic, NUMA, software and cooling. Peer-to-peer DMA excluded.</x:v>
+      </x:c>
+      <x:c r="T23" s="164"/>
+      <x:c r="U23" s="164"/>
+      <x:c r="V23" s="164"/>
+      <x:c r="W23" s="164"/>
+      <x:c r="X23" s="164"/>
+      <x:c r="Y23" s="164"/>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="S24" s="164" t="str">
+        <x:v>Software RAID0 (for example Linux md) can stripe visible NVMe block devices. Hardware/firmware RAID and boot support vary. RAID0 has no redundancy; a drive failure can lose the array.</x:v>
+      </x:c>
+      <x:c r="T24" s="164"/>
+      <x:c r="U24" s="164"/>
+      <x:c r="V24" s="164"/>
+      <x:c r="W24" s="164"/>
+      <x:c r="X24" s="164"/>
+      <x:c r="Y24" s="164"/>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="S25" s="164" t="str">
+        <x:v>Method sources: https://www.intel.com/content/www/us/en/gaming/resources/what-is-pcie-4-and-why-does-it-matter.html ; https://cdrdv2-public.intel.com/332995/332995-skl-io-platform-datasheet-vol1_rev004.pdf</x:v>
+      </x:c>
+      <x:c r="T25" s="164"/>
+      <x:c r="U25" s="164"/>
+      <x:c r="V25" s="164"/>
+      <x:c r="W25" s="164"/>
+      <x:c r="X25" s="164"/>
+      <x:c r="Y25" s="164"/>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="S26" s="164" t="str">
+        <x:v>Gen6 FLIT source: https://pcisig.com/blog/evolution-pci-express-specification-its-sixth-generation-third-decade-and-still-going-strong?PageSpeed=noscript ; RAID: https://docs.kernel.org/admin-guide/md.html</x:v>
+      </x:c>
+      <x:c r="T26" s="164"/>
+      <x:c r="U26" s="164"/>
+      <x:c r="V26" s="164"/>
+      <x:c r="W26" s="164"/>
+      <x:c r="X26" s="164"/>
+      <x:c r="Y26" s="164"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="S20:Y20"/>
+    <x:mergeCell ref="S21:Y21"/>
+    <x:mergeCell ref="S22:Y22"/>
+    <x:mergeCell ref="S23:Y23"/>
+    <x:mergeCell ref="S24:Y24"/>
+    <x:mergeCell ref="S25:Y25"/>
+    <x:mergeCell ref="S26:Y26"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7670795ad9794e9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b31cb24f7084660"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2204,7 +3367,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1e8223153d64cb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25b605d9950b4b46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2832,7 +3995,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2332afe8f90141f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0668e2d96c2a408b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3309,7 +4472,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bf345721c2748a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb457506d1c24271"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3708,7 +4871,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racaad3d6e1454441"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb33ed796049480e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4238,10 +5401,912 @@
         <x:v>Requires dedicated rack infrastructure and water cooling. Not a practical DIY cluster platform.</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="100" customHeight="1">
+      <x:c r="A14" s="102" t="str">
+        <x:v>Foxconn / Ampere</x:v>
+      </x:c>
+      <x:c r="B14" s="102" t="str">
+        <x:v>Mt. Collins 2U; dual Q80-30; 64GB</x:v>
+      </x:c>
+      <x:c r="C14" s="102" t="str">
+        <x:v>Used dual-socket 2U server</x:v>
+      </x:c>
+      <x:c r="D14" s="102" t="str">
+        <x:v>2x Altra Q80-30; 160 cores at 3.0 GHz</x:v>
+      </x:c>
+      <x:c r="E14" s="102" t="str">
+        <x:v>DDR4 ECC; 4x16GB DDR4-3200</x:v>
+      </x:c>
+      <x:c r="F14" s="103" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G14" s="104"/>
+      <x:c r="H14" s="102" t="str">
+        <x:v>4x25GbE SFP28 + 2x1GbE</x:v>
+      </x:c>
+      <x:c r="I14" s="102" t="str">
+        <x:v>PCIe Gen4; 24x U.2 NVMe bays</x:v>
+      </x:c>
+      <x:c r="J14" s="103"/>
+      <x:c r="K14" s="105" t="n">
+        <x:v>2200</x:v>
+      </x:c>
+      <x:c r="L14" s="102" t="str">
+        <x:v>Used private asking price; OBO</x:v>
+      </x:c>
+      <x:c r="M14" s="102" t="str">
+        <x:v>Seller repost; prior post says sold; verify</x:v>
+      </x:c>
+      <x:c r="N14" s="110" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="O14" s="107" t="n">
+        <x:f>IF(OR(F14="",F14=0),"",ROUNDUP(1024/F14,0))</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="P14" s="108" t="n">
+        <x:f>IF(OR(K14="",K14=0,O14=""),"",K14*O14)</x:f>
+        <x:v>35200</x:v>
+      </x:c>
+      <x:c r="Q14" s="109" t="str">
+        <x:v>Listing: https://www.reddit.com/r/homelabsales/comments/1wvbjd8/fsusnj_ampere_altra_foxconn_mt_collins_with_2/
+Platform: https://www.asacomputers.com/2u-24-bay-ampere-altra-arm-server.html?mode=spec</x:v>
+      </x:c>
+      <x:c r="R14" s="102" t="str">
+        <x:v>64GB and 1TB NVMe included. Local pickup only, Monmouth County NJ. Current repost asks $2,200; earlier post 1wl6t5y from same seller marks this configuration sold, so stock is unconfirmed. Four DIMMs do not populate all 16 CPU memory channels; bandwidth left blank. Dual 2000W PSUs are ratings, not system draw. 1-TiB cost repeats the listed 64GB system and excludes upgrades.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="100" customHeight="1">
+      <x:c r="A15" s="127" t="str">
+        <x:v>GIGABYTE</x:v>
+      </x:c>
+      <x:c r="B15" s="127" t="str">
+        <x:v>R272-P30-JG; Altra 80-core; 128GB</x:v>
+      </x:c>
+      <x:c r="C15" s="127" t="str">
+        <x:v>Used single-socket 2U server</x:v>
+      </x:c>
+      <x:c r="D15" s="127" t="str">
+        <x:v>1x Altra 80-core; 2.8 GHz listed; SKU unspecified</x:v>
+      </x:c>
+      <x:c r="E15" s="127" t="str">
+        <x:v>DDR4 ECC; 128GB installed</x:v>
+      </x:c>
+      <x:c r="F15" s="128" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="G15" s="129"/>
+      <x:c r="H15" s="127"/>
+      <x:c r="I15" s="127" t="str">
+        <x:v>NVMe storage; installed PCIe cards unspecified</x:v>
+      </x:c>
+      <x:c r="J15" s="128"/>
+      <x:c r="K15" s="130" t="n">
+        <x:v>3632</x:v>
+      </x:c>
+      <x:c r="L15" s="127" t="str">
+        <x:v>Historical used eBay displayed sold price</x:v>
+      </x:c>
+      <x:c r="M15" s="127" t="str">
+        <x:v>Sold 2026-07-14; historical reference</x:v>
+      </x:c>
+      <x:c r="N15" s="135" t="d">
+        <x:v>2026-07-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="O15" s="132" t="n">
+        <x:f>IF(OR(F15="",F15=0),"",ROUNDUP(1024/F15,0))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="P15" s="133" t="n">
+        <x:f>IF(OR(K15="",K15=0,O15=""),"",K15*O15)</x:f>
+        <x:v>29056</x:v>
+      </x:c>
+      <x:c r="Q15" s="134" t="str">
+        <x:v>Listing / configuration: https://www.ebay.com/itm/206345938406</x:v>
+      </x:c>
+      <x:c r="R15" s="127" t="str">
+        <x:v>Seller reports tested working. Includes 128GB Samsung DDR4 ECC, 2x7.68TB Micron 7300 PRO NVMe, and approximately 960GB Samsung M.2 NVMe. Exact CPU SKU, DIMM layout/speed, NIC and system draw unverified; bandwidth blank. Sold listing is a historical market reference. Price checked 2026-10-18; excludes tax. 1-TiB cost uses installed RAM, not 4TB platform capacity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="100" customHeight="1">
+      <x:c r="A16" s="102" t="str">
+        <x:v>GIGABYTE</x:v>
+      </x:c>
+      <x:c r="B16" s="102" t="str">
+        <x:v>R272-P30; M128-30; 256GB / 24SFF</x:v>
+      </x:c>
+      <x:c r="C16" s="102" t="str">
+        <x:v>Used single-socket 2U server</x:v>
+      </x:c>
+      <x:c r="D16" s="102" t="str">
+        <x:v>1x Altra Max M128-30; 128 cores at 3.0 GHz</x:v>
+      </x:c>
+      <x:c r="E16" s="102" t="str">
+        <x:v>DDR4 ECC RDIMM; 16x16GB DDR4-2666</x:v>
+      </x:c>
+      <x:c r="F16" s="103" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G16" s="104"/>
+      <x:c r="H16" s="102"/>
+      <x:c r="I16" s="102" t="str">
+        <x:v>4x CNV3122 NVMe adapters; 2x CNV3124 controllers</x:v>
+      </x:c>
+      <x:c r="J16" s="103"/>
+      <x:c r="K16" s="105" t="n">
+        <x:v>4999</x:v>
+      </x:c>
+      <x:c r="L16" s="102" t="str">
+        <x:v>Historical used eBay asking price; OBO</x:v>
+      </x:c>
+      <x:c r="M16" s="102" t="str">
+        <x:v>Ended 2026-07-24; unavailable</x:v>
+      </x:c>
+      <x:c r="N16" s="110" t="d">
+        <x:v>2026-07-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="O16" s="107" t="n">
+        <x:f>IF(OR(F16="",F16=0),"",ROUNDUP(1024/F16,0))</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P16" s="108" t="n">
+        <x:f>IF(OR(K16="",K16=0,O16=""),"",K16*O16)</x:f>
+        <x:v>19996</x:v>
+      </x:c>
+      <x:c r="Q16" s="109" t="str">
+        <x:v>Listing: https://www.ebay.com/itm/137275545029
+Configuration: seller description linked from listing (M128-30, 16x16GB PC4-2666V, 960GB M.2)</x:v>
+      </x:c>
+      <x:c r="R16" s="102" t="str">
+        <x:v>Includes Samsung PM983 960GB M.2, 24x2.5-inch NVMe chassis and 3x CEPM080 backplanes; no rails. $100 shipping extra. Listing ended; $4,999 is the advertised price, not a confirmed transaction. 1200W PSU rating is not system draw; CPU TDP is 250W. Actual memory operating speed unverified; bandwidth blank. 1-TiB cost repeats 256GB configuration and excludes shipping/tax.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb38901d93dfe41a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69e5e367f6bd42e8"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="35" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="33" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="25" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="90" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="95" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="162"/>
+      <x:c r="B1" s="162"/>
+      <x:c r="C1" s="162"/>
+      <x:c r="D1" s="162"/>
+      <x:c r="E1" s="162"/>
+      <x:c r="F1" s="162"/>
+      <x:c r="G1" s="162"/>
+      <x:c r="H1" s="162"/>
+      <x:c r="I1" s="162"/>
+      <x:c r="J1" s="162"/>
+      <x:c r="K1" s="162"/>
+      <x:c r="L1" s="162"/>
+      <x:c r="M1" s="162"/>
+      <x:c r="N1" s="162"/>
+      <x:c r="O1" s="162"/>
+      <x:c r="P1" s="162"/>
+      <x:c r="Q1" s="162"/>
+      <x:c r="R1" s="162"/>
+      <x:c r="S1" s="162"/>
+      <x:c r="T1" s="162"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="165" t="str">
+        <x:v>SSD database</x:v>
+      </x:c>
+      <x:c r="B2" s="162"/>
+      <x:c r="C2" s="162"/>
+      <x:c r="D2" s="162"/>
+      <x:c r="E2" s="162"/>
+      <x:c r="F2" s="162"/>
+      <x:c r="G2" s="162"/>
+      <x:c r="H2" s="162"/>
+      <x:c r="I2" s="162"/>
+      <x:c r="J2" s="162"/>
+      <x:c r="K2" s="162"/>
+      <x:c r="L2" s="162"/>
+      <x:c r="M2" s="162"/>
+      <x:c r="N2" s="162"/>
+      <x:c r="O2" s="162"/>
+      <x:c r="P2" s="162"/>
+      <x:c r="Q2" s="162"/>
+      <x:c r="R2" s="162"/>
+      <x:c r="S2" s="162"/>
+      <x:c r="T2" s="162"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="166"/>
+      <x:c r="B3" s="166"/>
+      <x:c r="C3" s="166"/>
+      <x:c r="D3" s="166"/>
+      <x:c r="E3" s="166"/>
+      <x:c r="F3" s="166"/>
+      <x:c r="G3" s="166"/>
+      <x:c r="H3" s="166"/>
+      <x:c r="I3" s="166"/>
+      <x:c r="J3" s="166"/>
+      <x:c r="K3" s="166"/>
+      <x:c r="L3" s="166"/>
+      <x:c r="M3" s="166"/>
+      <x:c r="N3" s="166"/>
+      <x:c r="O3" s="166"/>
+      <x:c r="P3" s="166"/>
+      <x:c r="Q3" s="166"/>
+      <x:c r="R3" s="166"/>
+      <x:c r="S3" s="166"/>
+      <x:c r="T3" s="166"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="167" t="str">
+        <x:v>NVMe SSDs: new and used. Performance is manufacturer-rated, not a benchmark of the listed unit. Prices exclude tax, adapters and host systems.</x:v>
+      </x:c>
+      <x:c r="B4" s="167"/>
+      <x:c r="C4" s="167"/>
+      <x:c r="D4" s="167"/>
+      <x:c r="E4" s="167"/>
+      <x:c r="F4" s="167"/>
+      <x:c r="G4" s="167"/>
+      <x:c r="H4" s="167"/>
+      <x:c r="I4" s="167"/>
+      <x:c r="J4" s="167"/>
+      <x:c r="K4" s="167"/>
+      <x:c r="L4" s="167"/>
+      <x:c r="M4" s="167"/>
+      <x:c r="N4" s="167"/>
+      <x:c r="O4" s="167"/>
+      <x:c r="P4" s="167"/>
+      <x:c r="Q4" s="167"/>
+      <x:c r="R4" s="167"/>
+      <x:c r="S4" s="167"/>
+      <x:c r="T4" s="167"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="162"/>
+      <x:c r="B5" s="162"/>
+      <x:c r="C5" s="162"/>
+      <x:c r="D5" s="162"/>
+      <x:c r="E5" s="162"/>
+      <x:c r="F5" s="162"/>
+      <x:c r="G5" s="162"/>
+      <x:c r="H5" s="162"/>
+      <x:c r="I5" s="162"/>
+      <x:c r="J5" s="162"/>
+      <x:c r="K5" s="162"/>
+      <x:c r="L5" s="162"/>
+      <x:c r="M5" s="162"/>
+      <x:c r="N5" s="162"/>
+      <x:c r="O5" s="162"/>
+      <x:c r="P5" s="162"/>
+      <x:c r="Q5" s="162"/>
+      <x:c r="R5" s="162"/>
+      <x:c r="S5" s="162"/>
+      <x:c r="T5" s="162"/>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="172" t="str">
+        <x:v>Vendor</x:v>
+      </x:c>
+      <x:c r="B6" s="172" t="str">
+        <x:v>Model / part number</x:v>
+      </x:c>
+      <x:c r="C6" s="172" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="D6" s="172" t="str">
+        <x:v>Capacity (TB; decimal)</x:v>
+      </x:c>
+      <x:c r="E6" s="172" t="str">
+        <x:v>Form factor</x:v>
+      </x:c>
+      <x:c r="F6" s="172" t="str">
+        <x:v>PCIe generation</x:v>
+      </x:c>
+      <x:c r="G6" s="172" t="str">
+        <x:v>PCIe lanes</x:v>
+      </x:c>
+      <x:c r="H6" s="172" t="str">
+        <x:v>Seq. read up to (MB/s)</x:v>
+      </x:c>
+      <x:c r="I6" s="172" t="str">
+        <x:v>Seq. write up to (MB/s)</x:v>
+      </x:c>
+      <x:c r="J6" s="172" t="str">
+        <x:v>Rated endurance (TBW)</x:v>
+      </x:c>
+      <x:c r="K6" s="172" t="str">
+        <x:v>Power-loss protection</x:v>
+      </x:c>
+      <x:c r="L6" s="172" t="str">
+        <x:v>Price (USD)</x:v>
+      </x:c>
+      <x:c r="M6" s="172" t="str">
+        <x:v>Price basis / seller</x:v>
+      </x:c>
+      <x:c r="N6" s="172" t="str">
+        <x:v>Availability</x:v>
+      </x:c>
+      <x:c r="O6" s="172" t="str">
+        <x:v>Price date</x:v>
+      </x:c>
+      <x:c r="P6" s="172" t="str">
+        <x:v>Price / TB (USD)</x:v>
+      </x:c>
+      <x:c r="Q6" s="172" t="str">
+        <x:v>4x RAID0 read (GB/s; ideal)</x:v>
+      </x:c>
+      <x:c r="R6" s="172" t="str">
+        <x:v>4x RAID0 write (GB/s; ideal)</x:v>
+      </x:c>
+      <x:c r="S6" s="172" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="T6" s="172" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" customHeight="1">
+      <x:c r="A7" s="175" t="str">
+        <x:v>Samsung</x:v>
+      </x:c>
+      <x:c r="B7" s="175" t="str">
+        <x:v>9100 PRO 4TB; MZ-VAP4T0B/AM</x:v>
+      </x:c>
+      <x:c r="C7" s="175" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D7" s="191" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="192" t="str">
+        <x:v>M.2 2280</x:v>
+      </x:c>
+      <x:c r="F7" s="193" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G7" s="193" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H7" s="193" t="n">
+        <x:v>14800</x:v>
+      </x:c>
+      <x:c r="I7" s="193" t="n">
+        <x:v>13400</x:v>
+      </x:c>
+      <x:c r="J7" s="193" t="n">
+        <x:v>2400</x:v>
+      </x:c>
+      <x:c r="K7" s="175" t="str">
+        <x:v>Enterprise PLP not specified</x:v>
+      </x:c>
+      <x:c r="L7" s="197" t="n">
+        <x:v>1049.95</x:v>
+      </x:c>
+      <x:c r="M7" s="175" t="str">
+        <x:v>Newegg marketplace / BioStar; asking</x:v>
+      </x:c>
+      <x:c r="N7" s="175" t="str">
+        <x:v>Listed; add to cart</x:v>
+      </x:c>
+      <x:c r="O7" s="189" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="P7" s="197" t="n">
+        <x:f>L7/D7</x:f>
+        <x:v>262.4875</x:v>
+      </x:c>
+      <x:c r="Q7" s="199" t="n">
+        <x:f>4*H7/1000</x:f>
+        <x:v>59.2</x:v>
+      </x:c>
+      <x:c r="R7" s="199" t="n">
+        <x:f>4*I7/1000</x:f>
+        <x:v>53.6</x:v>
+      </x:c>
+      <x:c r="S7" s="201" t="str">
+        <x:v>Specs: https://download.semiconductor.samsung.com/resources/data-sheet/Samsung_NVMe_SSD_9100_PRO_Datasheet_Rev.2.0.pdf
+Price: https://www.newegg.com/samsung-4tb-9100-pro-nvme-2-0/p/N82E16820147904</x:v>
+      </x:c>
+      <x:c r="T7" s="175" t="str">
+        <x:v>TLC consumer Gen5 drive, without heatsink. Vendor peak figures can use write cache; sustained writes after cache depletion can be much lower. Endurance is total rated writes, not remaining life. Active cooling/heatsink needed for long RAID workloads. Marketplace price is not MSRP.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" s="178" t="str">
+        <x:v>Sandisk / WD_BLACK</x:v>
+      </x:c>
+      <x:c r="B8" s="178" t="str">
+        <x:v>SN8100 4TB; WDS400T1X0M-00CMT0</x:v>
+      </x:c>
+      <x:c r="C8" s="178" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D8" s="194" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="195" t="str">
+        <x:v>M.2 2280</x:v>
+      </x:c>
+      <x:c r="F8" s="196" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G8" s="196" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H8" s="196" t="n">
+        <x:v>14900</x:v>
+      </x:c>
+      <x:c r="I8" s="196" t="n">
+        <x:v>14000</x:v>
+      </x:c>
+      <x:c r="J8" s="196" t="n">
+        <x:v>2400</x:v>
+      </x:c>
+      <x:c r="K8" s="178" t="str">
+        <x:v>Enterprise PLP not specified</x:v>
+      </x:c>
+      <x:c r="L8" s="198" t="n">
+        <x:v>839</x:v>
+      </x:c>
+      <x:c r="M8" s="178" t="str">
+        <x:v>Newegg marketplace / ShengYuan Parts Hub</x:v>
+      </x:c>
+      <x:c r="N8" s="178" t="str">
+        <x:v>Listed; ships from Hong Kong</x:v>
+      </x:c>
+      <x:c r="O8" s="190" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="P8" s="198" t="n">
+        <x:f>L8/D8</x:f>
+        <x:v>209.75</x:v>
+      </x:c>
+      <x:c r="Q8" s="200" t="n">
+        <x:f>4*H8/1000</x:f>
+        <x:v>59.6</x:v>
+      </x:c>
+      <x:c r="R8" s="200" t="n">
+        <x:f>4*I8/1000</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="S8" s="202" t="str">
+        <x:v>Specs: https://www.sandisk.com/en-ie/products/ssd/internal-ssd/wd-black-sn8100-ssd?sku=WDS400T1X0M-00CMT0
+Price: https://www.newegg.com/western-digital-4tb-nvme/p/N82E16820250280</x:v>
+      </x:c>
+      <x:c r="T8" s="178" t="str">
+        <x:v>TLC consumer Gen5 drive, without heatsink. Use manufacturer 4TB write rating (14,000 MB/s); retailer title says 11,000 MB/s. Consumer cache-assisted peaks are not sustained RAID performance. Verify exact SKU and seller warranty.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" s="175" t="str">
+        <x:v>Micron</x:v>
+      </x:c>
+      <x:c r="B9" s="175" t="str">
+        <x:v>9550 PRO 7.68TB; MTFDLAL7T6THA-1BK1JABYY</x:v>
+      </x:c>
+      <x:c r="C9" s="175" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D9" s="191" t="n">
+        <x:v>7.68</x:v>
+      </x:c>
+      <x:c r="E9" s="192" t="str">
+        <x:v>U.2 2.5-inch 15mm</x:v>
+      </x:c>
+      <x:c r="F9" s="193" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G9" s="193" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H9" s="193" t="n">
+        <x:v>14000</x:v>
+      </x:c>
+      <x:c r="I9" s="193" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="J9" s="193" t="n">
+        <x:v>14016</x:v>
+      </x:c>
+      <x:c r="K9" s="175" t="str">
+        <x:v>Yes; enterprise</x:v>
+      </x:c>
+      <x:c r="L9" s="197" t="n">
+        <x:v>8500</x:v>
+      </x:c>
+      <x:c r="M9" s="175" t="str">
+        <x:v>ServerSupply listed price; before checkout offers</x:v>
+      </x:c>
+      <x:c r="N9" s="175" t="str">
+        <x:v>Listed in stock</x:v>
+      </x:c>
+      <x:c r="O9" s="189" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="P9" s="197" t="n">
+        <x:f>L9/D9</x:f>
+        <x:v>1106.7708333333335</x:v>
+      </x:c>
+      <x:c r="Q9" s="199" t="n">
+        <x:f>4*H9/1000</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="R9" s="199" t="n">
+        <x:f>4*I9/1000</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="S9" s="201" t="str">
+        <x:v>Specs: https://tw.micron.com/content/dam/micron/global/public/products/product-flyer/9550-nvme-ssd-product-brief.pdf
+Price: https://www.serversupply.com/SSD/NVMe/7.68TB/MICRON/MTFDLAL7T6THA-1BK1JABYY_397182.htm</x:v>
+      </x:c>
+      <x:c r="T9" s="175" t="str">
+        <x:v>Enterprise TLC; 1 DWPD / 5 years; 14,016 TBW is 4K random endurance (sequential rating differs). Spec table is capacity-specific. Seller lists 90-day warranty and no manufacturer warranty. Price is one reseller observation, not a typical-market estimate. Requires a PCIe Gen5 NVMe U.2 path and airflow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10" s="178" t="str">
+        <x:v>Intel</x:v>
+      </x:c>
+      <x:c r="B10" s="178" t="str">
+        <x:v>Optane P5800X 1.6TB; SSDPF21Q016TB</x:v>
+      </x:c>
+      <x:c r="C10" s="178" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="D10" s="194" t="n">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="E10" s="195" t="str">
+        <x:v>U.2 2.5-inch 15mm</x:v>
+      </x:c>
+      <x:c r="F10" s="196" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G10" s="196" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H10" s="196" t="n">
+        <x:v>7200</x:v>
+      </x:c>
+      <x:c r="I10" s="196" t="n">
+        <x:v>6200</x:v>
+      </x:c>
+      <x:c r="J10" s="196" t="n">
+        <x:f>D10*100*365*5</x:f>
+        <x:v>292000</x:v>
+      </x:c>
+      <x:c r="K10" s="178" t="str">
+        <x:v>Yes; enhanced PLP</x:v>
+      </x:c>
+      <x:c r="L10" s="198" t="n">
+        <x:v>865</x:v>
+      </x:c>
+      <x:c r="M10" s="178" t="str">
+        <x:v>eBay / Long2207; asking; OBO</x:v>
+      </x:c>
+      <x:c r="N10" s="178" t="str">
+        <x:v>Listed 4 available; seller claim</x:v>
+      </x:c>
+      <x:c r="O10" s="190" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="P10" s="198" t="n">
+        <x:f>L10/D10</x:f>
+        <x:v>540.625</x:v>
+      </x:c>
+      <x:c r="Q10" s="200" t="n">
+        <x:f>4*H10/1000</x:f>
+        <x:v>28.8</x:v>
+      </x:c>
+      <x:c r="R10" s="200" t="n">
+        <x:f>4*I10/1000</x:f>
+        <x:v>24.8</x:v>
+      </x:c>
+      <x:c r="S10" s="202" t="str">
+        <x:v>Specs: https://www.intel.com/content/www/us/en/products/sku/201859/intel-optane-ssd-dc-p5800x-series-1-6tb-2-5in-pcie-x4-3d-xpoint/specifications.html
+Price: https://www.ebay.com/itm/800645585741</x:v>
+      </x:c>
+      <x:c r="T10" s="178" t="str">
+        <x:v>3D XPoint; high random-I/O/endurance option, not NAND TLC. Intel rates 1.5M random read/write IOPS and 100 DWPD over 5 years; TBW calculated from that rating. Seller claims 97–98% health; not independently verified. Obtain SMART/media-error/firmware data for the specific unit. Discontinued; warranty must be checked with seller.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="72" customHeight="1">
+      <x:c r="A11" s="175" t="str">
+        <x:v>Samsung</x:v>
+      </x:c>
+      <x:c r="B11" s="175" t="str">
+        <x:v>PM1733 7.68TB; MZWLJ7T6HALA-0007C</x:v>
+      </x:c>
+      <x:c r="C11" s="175" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="D11" s="191" t="n">
+        <x:v>7.68</x:v>
+      </x:c>
+      <x:c r="E11" s="192" t="str">
+        <x:v>U.2 2.5-inch 15mm</x:v>
+      </x:c>
+      <x:c r="F11" s="193" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G11" s="193" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H11" s="193" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="I11" s="193" t="n">
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="J11" s="193" t="n">
+        <x:f>D11*365*5</x:f>
+        <x:v>14016</x:v>
+      </x:c>
+      <x:c r="K11" s="175" t="str">
+        <x:v>Yes; enterprise</x:v>
+      </x:c>
+      <x:c r="L11" s="197" t="n">
+        <x:v>623.28</x:v>
+      </x:c>
+      <x:c r="M11" s="175" t="str">
+        <x:v>Historical eBay displayed sold price / tugm4470</x:v>
+      </x:c>
+      <x:c r="N11" s="175" t="str">
+        <x:v>Sold 2026-06-30; out of stock</x:v>
+      </x:c>
+      <x:c r="O11" s="189" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="P11" s="197" t="n">
+        <x:f>L11/D11</x:f>
+        <x:v>81.15625</x:v>
+      </x:c>
+      <x:c r="Q11" s="199" t="n">
+        <x:f>4*H11/1000</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="R11" s="199" t="n">
+        <x:f>4*I11/1000</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="S11" s="201" t="str">
+        <x:v>Specs: https://download.semiconductor.samsung.com/resources/brochure/PM1733%20NVMe%20SSD.pdf
+OEM capacity specs: https://lenovopress.lenovo.com/lp1300-thinksystem-pm1733-entry-nvme-ssd
+Price: https://www.ebay.com/itm/176400987818</x:v>
+      </x:c>
+      <x:c r="T11" s="175" t="str">
+        <x:v>Historical used reference, checked 2026-10-18; not a current offer. Seller claimed 97% health. Conservative published PM1733 read/write ratings; OEM -0007C firmware can differ from reference/OEM-guide drives. Rated endurance calculated at 1 DWPD / 5 years, not remaining writes. Verify sector format, firmware and full x4 port operation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="72" customHeight="1">
+      <x:c r="A12" s="178" t="str">
+        <x:v>Intel / Dell EMC</x:v>
+      </x:c>
+      <x:c r="B12" s="178" t="str">
+        <x:v>DC P4610 6.4TB; SSDPE2KE064T8T / 92F30</x:v>
+      </x:c>
+      <x:c r="C12" s="178" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="D12" s="194" t="n">
+        <x:v>6.4</x:v>
+      </x:c>
+      <x:c r="E12" s="195" t="str">
+        <x:v>U.2 2.5-inch 15mm</x:v>
+      </x:c>
+      <x:c r="F12" s="196" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G12" s="196" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H12" s="196" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="I12" s="196" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="J12" s="196" t="n">
+        <x:v>36540</x:v>
+      </x:c>
+      <x:c r="K12" s="178" t="str">
+        <x:v>Yes; enhanced PLP</x:v>
+      </x:c>
+      <x:c r="L12" s="198" t="n">
+        <x:v>379.99</x:v>
+      </x:c>
+      <x:c r="M12" s="178" t="str">
+        <x:v>PC Server &amp; Parts listed used price</x:v>
+      </x:c>
+      <x:c r="N12" s="178" t="str">
+        <x:v>Out of stock</x:v>
+      </x:c>
+      <x:c r="O12" s="190" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="P12" s="198" t="n">
+        <x:f>L12/D12</x:f>
+        <x:v>59.3734375</x:v>
+      </x:c>
+      <x:c r="Q12" s="200" t="n">
+        <x:f>4*H12/1000</x:f>
+        <x:v>12.8</x:v>
+      </x:c>
+      <x:c r="R12" s="200" t="n">
+        <x:f>4*I12/1000</x:f>
+        <x:v>12.8</x:v>
+      </x:c>
+      <x:c r="S12" s="202" t="str">
+        <x:v>Specs: https://lenovopress.lenovo.com/lp1032-intel-p4610-mainstream-nvme-pcie-ssds
+Price: https://pcserverandparts.com/dell-emc-dc-p4610-6-4tb-nvme-2-5-used-u-2-ssd-ssdpe2ke064t8t-92f30/</x:v>
+      </x:c>
+      <x:c r="T12" s="178" t="str">
+        <x:v>Older enterprise TLC option: high write endurance, slower Gen3 sequential speeds. 36,540 TBW and performance are published 6.4TB family/OEM-guide ratings; Dell firmware may vary. Seller lists tested/inspected, 90-day warranty; remaining endurance not stated. Price unavailable for immediate purchase; stock must return.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="161" t="str">
+        <x:v>Reading the comparison</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="A15" s="205" t="str">
+        <x:v>Units: capacity is decimal TB (1 TB = 10^12 bytes); MB/s and GB/s are decimal. SSD capacity is storage, not CPU RAM. TBW is total original rated endurance, not remaining life or a transferable warranty.</x:v>
+      </x:c>
+      <x:c r="B15" s="205"/>
+      <x:c r="C15" s="205"/>
+      <x:c r="D15" s="205"/>
+      <x:c r="E15" s="205"/>
+      <x:c r="F15" s="205"/>
+      <x:c r="G15" s="205"/>
+      <x:c r="H15" s="205"/>
+      <x:c r="I15" s="205"/>
+      <x:c r="J15" s="205"/>
+      <x:c r="K15" s="205"/>
+      <x:c r="L15" s="205"/>
+      <x:c r="M15" s="205"/>
+      <x:c r="N15" s="205"/>
+      <x:c r="O15" s="205"/>
+      <x:c r="P15" s="205"/>
+      <x:c r="Q15" s="205"/>
+      <x:c r="R15" s="205"/>
+      <x:c r="S15" s="205"/>
+      <x:c r="T15" s="205"/>
+    </x:row>
+    <x:row r="16" ht="26" customHeight="1">
+      <x:c r="A16" s="205" t="str">
+        <x:v>Four-drive RAID0 columns sum four identical SSD published sequential rates (4 × MB/s ÷ 1000). They require 16 host PCIe lanes at the SSD generation with suitable adapters/backplane; cap results by the CPU PCIe/RAM ceiling and actual switch uplinks. No tested scaling is implied.</x:v>
+      </x:c>
+      <x:c r="B16" s="205"/>
+      <x:c r="C16" s="205"/>
+      <x:c r="D16" s="205"/>
+      <x:c r="E16" s="205"/>
+      <x:c r="F16" s="205"/>
+      <x:c r="G16" s="205"/>
+      <x:c r="H16" s="205"/>
+      <x:c r="I16" s="205"/>
+      <x:c r="J16" s="205"/>
+      <x:c r="K16" s="205"/>
+      <x:c r="L16" s="205"/>
+      <x:c r="M16" s="205"/>
+      <x:c r="N16" s="205"/>
+      <x:c r="O16" s="205"/>
+      <x:c r="P16" s="205"/>
+      <x:c r="Q16" s="205"/>
+      <x:c r="R16" s="205"/>
+      <x:c r="S16" s="205"/>
+      <x:c r="T16" s="205"/>
+    </x:row>
+    <x:row r="17" ht="26" customHeight="1">
+      <x:c r="A17" s="205" t="str">
+        <x:v>M.2 consumer writes can drop sharply after SLC cache depletion. Enterprise figures use different test conditions, so peak numbers are not directly comparable sustained-workload benchmarks. RAID0 has no redundancy.</x:v>
+      </x:c>
+      <x:c r="B17" s="205"/>
+      <x:c r="C17" s="205"/>
+      <x:c r="D17" s="205"/>
+      <x:c r="E17" s="205"/>
+      <x:c r="F17" s="205"/>
+      <x:c r="G17" s="205"/>
+      <x:c r="H17" s="205"/>
+      <x:c r="I17" s="205"/>
+      <x:c r="J17" s="205"/>
+      <x:c r="K17" s="205"/>
+      <x:c r="L17" s="205"/>
+      <x:c r="M17" s="205"/>
+      <x:c r="N17" s="205"/>
+      <x:c r="O17" s="205"/>
+      <x:c r="P17" s="205"/>
+      <x:c r="Q17" s="205"/>
+      <x:c r="R17" s="205"/>
+      <x:c r="S17" s="205"/>
+      <x:c r="T17" s="205"/>
+    </x:row>
+    <x:row r="18" ht="26" customHeight="1">
+      <x:c r="A18" s="205" t="str">
+        <x:v>Used prices apply to the linked seller/configuration and can disappear. Verify NVMe SMART, Percentage Used, media errors, power-on hours, sector size, firmware, cooling and physical connector compatibility; seller health percentages are claims, not our measurements.</x:v>
+      </x:c>
+      <x:c r="B18" s="205"/>
+      <x:c r="C18" s="205"/>
+      <x:c r="D18" s="205"/>
+      <x:c r="E18" s="205"/>
+      <x:c r="F18" s="205"/>
+      <x:c r="G18" s="205"/>
+      <x:c r="H18" s="205"/>
+      <x:c r="I18" s="205"/>
+      <x:c r="J18" s="205"/>
+      <x:c r="K18" s="205"/>
+      <x:c r="L18" s="205"/>
+      <x:c r="M18" s="205"/>
+      <x:c r="N18" s="205"/>
+      <x:c r="O18" s="205"/>
+      <x:c r="P18" s="205"/>
+      <x:c r="Q18" s="205"/>
+      <x:c r="R18" s="205"/>
+      <x:c r="S18" s="205"/>
+      <x:c r="T18" s="205"/>
+    </x:row>
+    <x:row r="19" ht="26" customHeight="1">
+      <x:c r="A19" s="205" t="str">
+        <x:v>Consumer PLP is marked not specified because no enterprise power-loss guarantee was found in the cited specs. U.2/U.3/EDSFF and SAS/SATA bays are not interchangeable without a compatible host path.</x:v>
+      </x:c>
+      <x:c r="B19" s="205"/>
+      <x:c r="C19" s="205"/>
+      <x:c r="D19" s="205"/>
+      <x:c r="E19" s="205"/>
+      <x:c r="F19" s="205"/>
+      <x:c r="G19" s="205"/>
+      <x:c r="H19" s="205"/>
+      <x:c r="I19" s="205"/>
+      <x:c r="J19" s="205"/>
+      <x:c r="K19" s="205"/>
+      <x:c r="L19" s="205"/>
+      <x:c r="M19" s="205"/>
+      <x:c r="N19" s="205"/>
+      <x:c r="O19" s="205"/>
+      <x:c r="P19" s="205"/>
+      <x:c r="Q19" s="205"/>
+      <x:c r="R19" s="205"/>
+      <x:c r="S19" s="205"/>
+      <x:c r="T19" s="205"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A4:T4"/>
+    <x:mergeCell ref="A15:T15"/>
+    <x:mergeCell ref="A16:T16"/>
+    <x:mergeCell ref="A17:T17"/>
+    <x:mergeCell ref="A18:T18"/>
+    <x:mergeCell ref="A19:T19"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa543652d3dd4423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>